<commit_message>
Giai đoạn 11.2: detail design Đăng nhập, Đổi mật khẩu, Khung ứng dụng, Tổng quan
- 01_DangNhap: ô nhập, ghi nhớ thiết bị, thông báo lỗi (sai mật khẩu, bị khoá, khoá tạm),
  xử lý ở backend, sơ đồ luồng đăng nhập.
- 02_DoiMatKhau: bắt đổi lần đầu, quy tắc mật khẩu, nhập lại không khớp, sai mật khẩu hiện tại.
- 03_KhungUngDung: menu, thanh trên, chuông và 4 loại thông báo (điều kiện, ai thấy, nút xử
  lý nhanh), dark mode, giao diện iPad, đăng xuất.
- 04_TongQuan: chỉ số hôm nay, thẻ phòng theo trạng thái, việc cần làm, doanh thu 7 ngày,
  cơ cấu đơn, công suất; khác biệt khi Nhân viên xem.
- Công cụ: chụp theo kích thước màn hình riêng (iPad) và context riêng (dark mode), thêm vị
  trí số đánh dấu; sinh lại 00_TongThe với cách tính chiều cao dòng mới.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/detail-design/00_TongThe.xlsx
+++ b/docs/detail-design/00_TongThe.xlsx
@@ -2509,7 +2509,7 @@
       <xdr:row>107</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="11182350" cy="8765365"/>
+    <xdr:ext cx="9658350" cy="7570767"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 2">
@@ -2553,7 +2553,7 @@
       <xdr:row>28</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="11182350" cy="3304905"/>
+    <xdr:ext cx="9658350" cy="2854492"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -5394,7 +5394,7 @@
       <c r="AF98" s="5"/>
       <c r="AG98" s="5"/>
     </row>
-    <row r="99" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B99" s="3" t="s">
         <v>131</v>
       </c>
@@ -6527,7 +6527,7 @@
       <c r="AF19" s="3"/>
       <c r="AG19" s="3"/>
     </row>
-    <row r="20" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B20" s="8">
         <v>15</v>
       </c>
@@ -6695,7 +6695,7 @@
       <c r="AF23" s="3"/>
       <c r="AG23" s="3"/>
     </row>
-    <row r="24" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B24" s="8">
         <v>19</v>
       </c>
@@ -19134,7 +19134,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AG130"/>
+  <dimension ref="B1:AG127"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -19327,7 +19327,7 @@
       <c r="AF5" s="7"/>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" ht="43" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="6" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
         <v>521</v>
       </c>
@@ -19629,7 +19629,7 @@
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
     </row>
-    <row r="15" ht="56" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="15" ht="43" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>536</v>
       </c>
@@ -20087,58 +20087,184 @@
       <c r="AF28" s="6"/>
       <c r="AG28" s="6"/>
     </row>
-    <row r="48" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B48" s="5" t="s">
+    <row r="45" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B45" s="5" t="s">
         <v>561</v>
       </c>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5" t="s">
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5" t="s">
         <v>562</v>
       </c>
-      <c r="H48" s="5"/>
-      <c r="I48" s="5"/>
-      <c r="J48" s="5"/>
-      <c r="K48" s="5"/>
-      <c r="L48" s="5"/>
-      <c r="M48" s="5"/>
-      <c r="N48" s="5"/>
-      <c r="O48" s="5"/>
-      <c r="P48" s="5" t="s">
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="K45" s="5"/>
+      <c r="L45" s="5"/>
+      <c r="M45" s="5"/>
+      <c r="N45" s="5"/>
+      <c r="O45" s="5"/>
+      <c r="P45" s="5" t="s">
         <v>563</v>
       </c>
-      <c r="Q48" s="5"/>
-      <c r="R48" s="5"/>
-      <c r="S48" s="5"/>
-      <c r="T48" s="5"/>
-      <c r="U48" s="5"/>
-      <c r="V48" s="5"/>
-      <c r="W48" s="5" t="s">
+      <c r="Q45" s="5"/>
+      <c r="R45" s="5"/>
+      <c r="S45" s="5"/>
+      <c r="T45" s="5"/>
+      <c r="U45" s="5"/>
+      <c r="V45" s="5"/>
+      <c r="W45" s="5" t="s">
         <v>564</v>
       </c>
-      <c r="X48" s="5"/>
-      <c r="Y48" s="5"/>
-      <c r="Z48" s="5"/>
-      <c r="AA48" s="5"/>
-      <c r="AB48" s="5"/>
-      <c r="AC48" s="5"/>
-      <c r="AD48" s="5"/>
-      <c r="AE48" s="5"/>
-      <c r="AF48" s="5"/>
-      <c r="AG48" s="5"/>
-    </row>
-    <row r="49" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="X45" s="5"/>
+      <c r="Y45" s="5"/>
+      <c r="Z45" s="5"/>
+      <c r="AA45" s="5"/>
+      <c r="AB45" s="5"/>
+      <c r="AC45" s="5"/>
+      <c r="AD45" s="5"/>
+      <c r="AE45" s="5"/>
+      <c r="AF45" s="5"/>
+      <c r="AG45" s="5"/>
+    </row>
+    <row r="46" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B46" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
+      <c r="N46" s="3"/>
+      <c r="O46" s="3"/>
+      <c r="P46" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="Q46" s="3"/>
+      <c r="R46" s="3"/>
+      <c r="S46" s="3"/>
+      <c r="T46" s="3"/>
+      <c r="U46" s="3"/>
+      <c r="V46" s="3"/>
+      <c r="W46" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="X46" s="3"/>
+      <c r="Y46" s="3"/>
+      <c r="Z46" s="3"/>
+      <c r="AA46" s="3"/>
+      <c r="AB46" s="3"/>
+      <c r="AC46" s="3"/>
+      <c r="AD46" s="3"/>
+      <c r="AE46" s="3"/>
+      <c r="AF46" s="3"/>
+      <c r="AG46" s="3"/>
+    </row>
+    <row r="47" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B47" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+      <c r="N47" s="3"/>
+      <c r="O47" s="3"/>
+      <c r="P47" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="Q47" s="3"/>
+      <c r="R47" s="3"/>
+      <c r="S47" s="3"/>
+      <c r="T47" s="3"/>
+      <c r="U47" s="3"/>
+      <c r="V47" s="3"/>
+      <c r="W47" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="X47" s="3"/>
+      <c r="Y47" s="3"/>
+      <c r="Z47" s="3"/>
+      <c r="AA47" s="3"/>
+      <c r="AB47" s="3"/>
+      <c r="AC47" s="3"/>
+      <c r="AD47" s="3"/>
+      <c r="AE47" s="3"/>
+      <c r="AF47" s="3"/>
+      <c r="AG47" s="3"/>
+    </row>
+    <row r="48" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B48" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="3"/>
+      <c r="P48" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="Q48" s="3"/>
+      <c r="R48" s="3"/>
+      <c r="S48" s="3"/>
+      <c r="T48" s="3"/>
+      <c r="U48" s="3"/>
+      <c r="V48" s="3"/>
+      <c r="W48" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="X48" s="3"/>
+      <c r="Y48" s="3"/>
+      <c r="Z48" s="3"/>
+      <c r="AA48" s="3"/>
+      <c r="AB48" s="3"/>
+      <c r="AC48" s="3"/>
+      <c r="AD48" s="3"/>
+      <c r="AE48" s="3"/>
+      <c r="AF48" s="3"/>
+      <c r="AG48" s="3"/>
+    </row>
+    <row r="49" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B49" s="3" t="s">
-        <v>565</v>
+        <v>576</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
       <c r="G49" s="3" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
@@ -20149,7 +20275,7 @@
       <c r="N49" s="3"/>
       <c r="O49" s="3"/>
       <c r="P49" s="3" t="s">
-        <v>567</v>
+        <v>578</v>
       </c>
       <c r="Q49" s="3"/>
       <c r="R49" s="3"/>
@@ -20158,7 +20284,7 @@
       <c r="U49" s="3"/>
       <c r="V49" s="3"/>
       <c r="W49" s="3" t="s">
-        <v>568</v>
+        <v>579</v>
       </c>
       <c r="X49" s="3"/>
       <c r="Y49" s="3"/>
@@ -20173,14 +20299,14 @@
     </row>
     <row r="50" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B50" s="3" t="s">
-        <v>569</v>
+        <v>580</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
       <c r="G50" s="3" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="H50" s="3"/>
       <c r="I50" s="3"/>
@@ -20191,7 +20317,7 @@
       <c r="N50" s="3"/>
       <c r="O50" s="3"/>
       <c r="P50" s="3" t="s">
-        <v>571</v>
+        <v>581</v>
       </c>
       <c r="Q50" s="3"/>
       <c r="R50" s="3"/>
@@ -20200,7 +20326,7 @@
       <c r="U50" s="3"/>
       <c r="V50" s="3"/>
       <c r="W50" s="3" t="s">
-        <v>572</v>
+        <v>582</v>
       </c>
       <c r="X50" s="3"/>
       <c r="Y50" s="3"/>
@@ -20215,14 +20341,14 @@
     </row>
     <row r="51" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B51" s="3" t="s">
-        <v>573</v>
+        <v>583</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
       <c r="G51" s="3" t="s">
-        <v>570</v>
+        <v>584</v>
       </c>
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
@@ -20233,7 +20359,7 @@
       <c r="N51" s="3"/>
       <c r="O51" s="3"/>
       <c r="P51" s="3" t="s">
-        <v>574</v>
+        <v>585</v>
       </c>
       <c r="Q51" s="3"/>
       <c r="R51" s="3"/>
@@ -20242,7 +20368,7 @@
       <c r="U51" s="3"/>
       <c r="V51" s="3"/>
       <c r="W51" s="3" t="s">
-        <v>575</v>
+        <v>586</v>
       </c>
       <c r="X51" s="3"/>
       <c r="Y51" s="3"/>
@@ -20255,211 +20381,205 @@
       <c r="AF51" s="3"/>
       <c r="AG51" s="3"/>
     </row>
-    <row r="52" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B52" s="3" t="s">
-        <v>576</v>
-      </c>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="3" t="s">
-        <v>577</v>
-      </c>
-      <c r="H52" s="3"/>
-      <c r="I52" s="3"/>
-      <c r="J52" s="3"/>
-      <c r="K52" s="3"/>
-      <c r="L52" s="3"/>
-      <c r="M52" s="3"/>
-      <c r="N52" s="3"/>
-      <c r="O52" s="3"/>
-      <c r="P52" s="3" t="s">
-        <v>578</v>
-      </c>
-      <c r="Q52" s="3"/>
-      <c r="R52" s="3"/>
-      <c r="S52" s="3"/>
-      <c r="T52" s="3"/>
-      <c r="U52" s="3"/>
-      <c r="V52" s="3"/>
-      <c r="W52" s="3" t="s">
-        <v>579</v>
-      </c>
-      <c r="X52" s="3"/>
-      <c r="Y52" s="3"/>
-      <c r="Z52" s="3"/>
-      <c r="AA52" s="3"/>
-      <c r="AB52" s="3"/>
-      <c r="AC52" s="3"/>
-      <c r="AD52" s="3"/>
-      <c r="AE52" s="3"/>
-      <c r="AF52" s="3"/>
-      <c r="AG52" s="3"/>
-    </row>
-    <row r="53" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B53" s="3" t="s">
-        <v>580</v>
-      </c>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3" t="s">
-        <v>566</v>
-      </c>
-      <c r="H53" s="3"/>
-      <c r="I53" s="3"/>
-      <c r="J53" s="3"/>
-      <c r="K53" s="3"/>
-      <c r="L53" s="3"/>
-      <c r="M53" s="3"/>
-      <c r="N53" s="3"/>
-      <c r="O53" s="3"/>
-      <c r="P53" s="3" t="s">
-        <v>581</v>
-      </c>
-      <c r="Q53" s="3"/>
-      <c r="R53" s="3"/>
-      <c r="S53" s="3"/>
-      <c r="T53" s="3"/>
-      <c r="U53" s="3"/>
-      <c r="V53" s="3"/>
-      <c r="W53" s="3" t="s">
-        <v>582</v>
-      </c>
-      <c r="X53" s="3"/>
-      <c r="Y53" s="3"/>
-      <c r="Z53" s="3"/>
-      <c r="AA53" s="3"/>
-      <c r="AB53" s="3"/>
-      <c r="AC53" s="3"/>
-      <c r="AD53" s="3"/>
-      <c r="AE53" s="3"/>
-      <c r="AF53" s="3"/>
-      <c r="AG53" s="3"/>
-    </row>
-    <row r="54" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B54" s="3" t="s">
-        <v>583</v>
-      </c>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="3" t="s">
-        <v>584</v>
-      </c>
-      <c r="H54" s="3"/>
-      <c r="I54" s="3"/>
-      <c r="J54" s="3"/>
-      <c r="K54" s="3"/>
-      <c r="L54" s="3"/>
-      <c r="M54" s="3"/>
-      <c r="N54" s="3"/>
-      <c r="O54" s="3"/>
-      <c r="P54" s="3" t="s">
-        <v>585</v>
-      </c>
-      <c r="Q54" s="3"/>
-      <c r="R54" s="3"/>
-      <c r="S54" s="3"/>
-      <c r="T54" s="3"/>
-      <c r="U54" s="3"/>
-      <c r="V54" s="3"/>
-      <c r="W54" s="3" t="s">
-        <v>586</v>
-      </c>
-      <c r="X54" s="3"/>
-      <c r="Y54" s="3"/>
-      <c r="Z54" s="3"/>
-      <c r="AA54" s="3"/>
-      <c r="AB54" s="3"/>
-      <c r="AC54" s="3"/>
-      <c r="AD54" s="3"/>
-      <c r="AE54" s="3"/>
-      <c r="AF54" s="3"/>
-      <c r="AG54" s="3"/>
-    </row>
-    <row r="56" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B56" s="4" t="s">
+    <row r="53" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B53" s="4" t="s">
         <v>587</v>
       </c>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
-      <c r="I56" s="4"/>
-      <c r="J56" s="4"/>
-      <c r="K56" s="4"/>
-      <c r="L56" s="4"/>
-      <c r="M56" s="4"/>
-      <c r="N56" s="4"/>
-      <c r="O56" s="4"/>
-      <c r="P56" s="4"/>
-      <c r="Q56" s="4"/>
-      <c r="R56" s="4"/>
-      <c r="S56" s="4"/>
-      <c r="T56" s="4"/>
-      <c r="U56" s="4"/>
-      <c r="V56" s="4"/>
-      <c r="W56" s="4"/>
-      <c r="X56" s="4"/>
-      <c r="Y56" s="4"/>
-      <c r="Z56" s="4"/>
-      <c r="AA56" s="4"/>
-      <c r="AB56" s="4"/>
-      <c r="AC56" s="4"/>
-      <c r="AD56" s="4"/>
-      <c r="AE56" s="4"/>
-      <c r="AF56" s="4"/>
-      <c r="AG56" s="4"/>
-    </row>
-    <row r="57" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B57" s="5" t="s">
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
+      <c r="I53" s="4"/>
+      <c r="J53" s="4"/>
+      <c r="K53" s="4"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4"/>
+      <c r="P53" s="4"/>
+      <c r="Q53" s="4"/>
+      <c r="R53" s="4"/>
+      <c r="S53" s="4"/>
+      <c r="T53" s="4"/>
+      <c r="U53" s="4"/>
+      <c r="V53" s="4"/>
+      <c r="W53" s="4"/>
+      <c r="X53" s="4"/>
+      <c r="Y53" s="4"/>
+      <c r="Z53" s="4"/>
+      <c r="AA53" s="4"/>
+      <c r="AB53" s="4"/>
+      <c r="AC53" s="4"/>
+      <c r="AD53" s="4"/>
+      <c r="AE53" s="4"/>
+      <c r="AF53" s="4"/>
+      <c r="AG53" s="4"/>
+    </row>
+    <row r="54" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B54" s="5" t="s">
         <v>485</v>
       </c>
-      <c r="C57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
-      <c r="G57" s="5"/>
-      <c r="H57" s="5"/>
-      <c r="I57" s="5" t="s">
+      <c r="C54" s="5"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="J57" s="5"/>
-      <c r="K57" s="5"/>
-      <c r="L57" s="5"/>
-      <c r="M57" s="5"/>
-      <c r="N57" s="5"/>
-      <c r="O57" s="5"/>
-      <c r="P57" s="5"/>
-      <c r="Q57" s="5"/>
-      <c r="R57" s="5"/>
-      <c r="S57" s="5"/>
-      <c r="T57" s="5"/>
-      <c r="U57" s="5"/>
-      <c r="V57" s="5"/>
-      <c r="W57" s="5"/>
-      <c r="X57" s="5" t="s">
+      <c r="J54" s="5"/>
+      <c r="K54" s="5"/>
+      <c r="L54" s="5"/>
+      <c r="M54" s="5"/>
+      <c r="N54" s="5"/>
+      <c r="O54" s="5"/>
+      <c r="P54" s="5"/>
+      <c r="Q54" s="5"/>
+      <c r="R54" s="5"/>
+      <c r="S54" s="5"/>
+      <c r="T54" s="5"/>
+      <c r="U54" s="5"/>
+      <c r="V54" s="5"/>
+      <c r="W54" s="5"/>
+      <c r="X54" s="5" t="s">
         <v>589</v>
       </c>
-      <c r="Y57" s="5"/>
-      <c r="Z57" s="5"/>
-      <c r="AA57" s="5"/>
-      <c r="AB57" s="5"/>
-      <c r="AC57" s="5"/>
-      <c r="AD57" s="5"/>
-      <c r="AE57" s="5"/>
-      <c r="AF57" s="5"/>
-      <c r="AG57" s="5"/>
+      <c r="Y54" s="5"/>
+      <c r="Z54" s="5"/>
+      <c r="AA54" s="5"/>
+      <c r="AB54" s="5"/>
+      <c r="AC54" s="5"/>
+      <c r="AD54" s="5"/>
+      <c r="AE54" s="5"/>
+      <c r="AF54" s="5"/>
+      <c r="AG54" s="5"/>
+    </row>
+    <row r="55" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B55" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="J55" s="3"/>
+      <c r="K55" s="3"/>
+      <c r="L55" s="3"/>
+      <c r="M55" s="3"/>
+      <c r="N55" s="3"/>
+      <c r="O55" s="3"/>
+      <c r="P55" s="3"/>
+      <c r="Q55" s="3"/>
+      <c r="R55" s="3"/>
+      <c r="S55" s="3"/>
+      <c r="T55" s="3"/>
+      <c r="U55" s="3"/>
+      <c r="V55" s="3"/>
+      <c r="W55" s="3"/>
+      <c r="X55" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="Y55" s="3"/>
+      <c r="Z55" s="3"/>
+      <c r="AA55" s="3"/>
+      <c r="AB55" s="3"/>
+      <c r="AC55" s="3"/>
+      <c r="AD55" s="3"/>
+      <c r="AE55" s="3"/>
+      <c r="AF55" s="3"/>
+      <c r="AG55" s="3"/>
+    </row>
+    <row r="56" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B56" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="J56" s="3"/>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="3"/>
+      <c r="N56" s="3"/>
+      <c r="O56" s="3"/>
+      <c r="P56" s="3"/>
+      <c r="Q56" s="3"/>
+      <c r="R56" s="3"/>
+      <c r="S56" s="3"/>
+      <c r="T56" s="3"/>
+      <c r="U56" s="3"/>
+      <c r="V56" s="3"/>
+      <c r="W56" s="3"/>
+      <c r="X56" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="Y56" s="3"/>
+      <c r="Z56" s="3"/>
+      <c r="AA56" s="3"/>
+      <c r="AB56" s="3"/>
+      <c r="AC56" s="3"/>
+      <c r="AD56" s="3"/>
+      <c r="AE56" s="3"/>
+      <c r="AF56" s="3"/>
+      <c r="AG56" s="3"/>
+    </row>
+    <row r="57" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B57" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="J57" s="3"/>
+      <c r="K57" s="3"/>
+      <c r="L57" s="3"/>
+      <c r="M57" s="3"/>
+      <c r="N57" s="3"/>
+      <c r="O57" s="3"/>
+      <c r="P57" s="3"/>
+      <c r="Q57" s="3"/>
+      <c r="R57" s="3"/>
+      <c r="S57" s="3"/>
+      <c r="T57" s="3"/>
+      <c r="U57" s="3"/>
+      <c r="V57" s="3"/>
+      <c r="W57" s="3"/>
+      <c r="X57" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="Y57" s="3"/>
+      <c r="Z57" s="3"/>
+      <c r="AA57" s="3"/>
+      <c r="AB57" s="3"/>
+      <c r="AC57" s="3"/>
+      <c r="AD57" s="3"/>
+      <c r="AE57" s="3"/>
+      <c r="AF57" s="3"/>
+      <c r="AG57" s="3"/>
     </row>
     <row r="58" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B58" s="3" t="s">
-        <v>590</v>
+        <v>599</v>
       </c>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
@@ -20468,7 +20588,7 @@
       <c r="G58" s="3"/>
       <c r="H58" s="3"/>
       <c r="I58" s="3" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="J58" s="3"/>
       <c r="K58" s="3"/>
@@ -20485,7 +20605,7 @@
       <c r="V58" s="3"/>
       <c r="W58" s="3"/>
       <c r="X58" s="3" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="Y58" s="3"/>
       <c r="Z58" s="3"/>
@@ -20499,7 +20619,7 @@
     </row>
     <row r="59" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B59" s="3" t="s">
-        <v>593</v>
+        <v>601</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
@@ -20508,7 +20628,7 @@
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
       <c r="I59" s="3" t="s">
-        <v>594</v>
+        <v>602</v>
       </c>
       <c r="J59" s="3"/>
       <c r="K59" s="3"/>
@@ -20525,7 +20645,7 @@
       <c r="V59" s="3"/>
       <c r="W59" s="3"/>
       <c r="X59" s="3" t="s">
-        <v>595</v>
+        <v>603</v>
       </c>
       <c r="Y59" s="3"/>
       <c r="Z59" s="3"/>
@@ -20537,9 +20657,9 @@
       <c r="AF59" s="3"/>
       <c r="AG59" s="3"/>
     </row>
-    <row r="60" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B60" s="3" t="s">
-        <v>596</v>
+        <v>604</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
@@ -20548,7 +20668,7 @@
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
       <c r="I60" s="3" t="s">
-        <v>597</v>
+        <v>605</v>
       </c>
       <c r="J60" s="3"/>
       <c r="K60" s="3"/>
@@ -20565,7 +20685,7 @@
       <c r="V60" s="3"/>
       <c r="W60" s="3"/>
       <c r="X60" s="3" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="Y60" s="3"/>
       <c r="Z60" s="3"/>
@@ -20579,7 +20699,7 @@
     </row>
     <row r="61" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B61" s="3" t="s">
-        <v>599</v>
+        <v>606</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
@@ -20588,7 +20708,7 @@
       <c r="G61" s="3"/>
       <c r="H61" s="3"/>
       <c r="I61" s="3" t="s">
-        <v>600</v>
+        <v>607</v>
       </c>
       <c r="J61" s="3"/>
       <c r="K61" s="3"/>
@@ -20605,7 +20725,7 @@
       <c r="V61" s="3"/>
       <c r="W61" s="3"/>
       <c r="X61" s="3" t="s">
-        <v>595</v>
+        <v>608</v>
       </c>
       <c r="Y61" s="3"/>
       <c r="Z61" s="3"/>
@@ -20617,9 +20737,9 @@
       <c r="AF61" s="3"/>
       <c r="AG61" s="3"/>
     </row>
-    <row r="62" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="62" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B62" s="3" t="s">
-        <v>601</v>
+        <v>609</v>
       </c>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
@@ -20628,7 +20748,7 @@
       <c r="G62" s="3"/>
       <c r="H62" s="3"/>
       <c r="I62" s="3" t="s">
-        <v>602</v>
+        <v>610</v>
       </c>
       <c r="J62" s="3"/>
       <c r="K62" s="3"/>
@@ -20645,7 +20765,7 @@
       <c r="V62" s="3"/>
       <c r="W62" s="3"/>
       <c r="X62" s="3" t="s">
-        <v>603</v>
+        <v>592</v>
       </c>
       <c r="Y62" s="3"/>
       <c r="Z62" s="3"/>
@@ -20659,7 +20779,7 @@
     </row>
     <row r="63" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B63" s="3" t="s">
-        <v>604</v>
+        <v>611</v>
       </c>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
@@ -20668,7 +20788,7 @@
       <c r="G63" s="3"/>
       <c r="H63" s="3"/>
       <c r="I63" s="3" t="s">
-        <v>605</v>
+        <v>612</v>
       </c>
       <c r="J63" s="3"/>
       <c r="K63" s="3"/>
@@ -20685,7 +20805,7 @@
       <c r="V63" s="3"/>
       <c r="W63" s="3"/>
       <c r="X63" s="3" t="s">
-        <v>595</v>
+        <v>613</v>
       </c>
       <c r="Y63" s="3"/>
       <c r="Z63" s="3"/>
@@ -20697,254 +20817,272 @@
       <c r="AF63" s="3"/>
       <c r="AG63" s="3"/>
     </row>
-    <row r="64" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B64" s="3" t="s">
-        <v>606</v>
-      </c>
-      <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
-      <c r="E64" s="3"/>
-      <c r="F64" s="3"/>
-      <c r="G64" s="3"/>
-      <c r="H64" s="3"/>
-      <c r="I64" s="3" t="s">
-        <v>607</v>
-      </c>
-      <c r="J64" s="3"/>
-      <c r="K64" s="3"/>
-      <c r="L64" s="3"/>
-      <c r="M64" s="3"/>
-      <c r="N64" s="3"/>
-      <c r="O64" s="3"/>
-      <c r="P64" s="3"/>
-      <c r="Q64" s="3"/>
-      <c r="R64" s="3"/>
-      <c r="S64" s="3"/>
-      <c r="T64" s="3"/>
-      <c r="U64" s="3"/>
-      <c r="V64" s="3"/>
-      <c r="W64" s="3"/>
-      <c r="X64" s="3" t="s">
-        <v>608</v>
-      </c>
-      <c r="Y64" s="3"/>
-      <c r="Z64" s="3"/>
-      <c r="AA64" s="3"/>
-      <c r="AB64" s="3"/>
-      <c r="AC64" s="3"/>
-      <c r="AD64" s="3"/>
-      <c r="AE64" s="3"/>
-      <c r="AF64" s="3"/>
-      <c r="AG64" s="3"/>
-    </row>
-    <row r="65" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B65" s="3" t="s">
-        <v>609</v>
-      </c>
-      <c r="C65" s="3"/>
-      <c r="D65" s="3"/>
-      <c r="E65" s="3"/>
-      <c r="F65" s="3"/>
-      <c r="G65" s="3"/>
-      <c r="H65" s="3"/>
-      <c r="I65" s="3" t="s">
-        <v>610</v>
-      </c>
-      <c r="J65" s="3"/>
-      <c r="K65" s="3"/>
-      <c r="L65" s="3"/>
-      <c r="M65" s="3"/>
-      <c r="N65" s="3"/>
-      <c r="O65" s="3"/>
-      <c r="P65" s="3"/>
-      <c r="Q65" s="3"/>
-      <c r="R65" s="3"/>
-      <c r="S65" s="3"/>
-      <c r="T65" s="3"/>
-      <c r="U65" s="3"/>
-      <c r="V65" s="3"/>
-      <c r="W65" s="3"/>
-      <c r="X65" s="3" t="s">
-        <v>592</v>
-      </c>
-      <c r="Y65" s="3"/>
-      <c r="Z65" s="3"/>
-      <c r="AA65" s="3"/>
-      <c r="AB65" s="3"/>
-      <c r="AC65" s="3"/>
-      <c r="AD65" s="3"/>
-      <c r="AE65" s="3"/>
-      <c r="AF65" s="3"/>
-      <c r="AG65" s="3"/>
-    </row>
-    <row r="66" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B66" s="3" t="s">
-        <v>611</v>
-      </c>
-      <c r="C66" s="3"/>
-      <c r="D66" s="3"/>
-      <c r="E66" s="3"/>
-      <c r="F66" s="3"/>
-      <c r="G66" s="3"/>
-      <c r="H66" s="3"/>
-      <c r="I66" s="3" t="s">
-        <v>612</v>
-      </c>
-      <c r="J66" s="3"/>
-      <c r="K66" s="3"/>
-      <c r="L66" s="3"/>
-      <c r="M66" s="3"/>
-      <c r="N66" s="3"/>
-      <c r="O66" s="3"/>
-      <c r="P66" s="3"/>
-      <c r="Q66" s="3"/>
-      <c r="R66" s="3"/>
-      <c r="S66" s="3"/>
-      <c r="T66" s="3"/>
-      <c r="U66" s="3"/>
-      <c r="V66" s="3"/>
-      <c r="W66" s="3"/>
-      <c r="X66" s="3" t="s">
-        <v>613</v>
-      </c>
-      <c r="Y66" s="3"/>
-      <c r="Z66" s="3"/>
-      <c r="AA66" s="3"/>
-      <c r="AB66" s="3"/>
-      <c r="AC66" s="3"/>
-      <c r="AD66" s="3"/>
-      <c r="AE66" s="3"/>
-      <c r="AF66" s="3"/>
-      <c r="AG66" s="3"/>
-    </row>
-    <row r="67" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B67" s="6" t="s">
+    <row r="64" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B64" s="6" t="s">
         <v>614</v>
       </c>
-      <c r="C67" s="6"/>
-      <c r="D67" s="6"/>
-      <c r="E67" s="6"/>
-      <c r="F67" s="6"/>
-      <c r="G67" s="6"/>
-      <c r="H67" s="6"/>
-      <c r="I67" s="6"/>
-      <c r="J67" s="6"/>
-      <c r="K67" s="6"/>
-      <c r="L67" s="6"/>
-      <c r="M67" s="6"/>
-      <c r="N67" s="6"/>
-      <c r="O67" s="6"/>
-      <c r="P67" s="6"/>
-      <c r="Q67" s="6"/>
-      <c r="R67" s="6"/>
-      <c r="S67" s="6"/>
-      <c r="T67" s="6"/>
-      <c r="U67" s="6"/>
-      <c r="V67" s="6"/>
-      <c r="W67" s="6"/>
-      <c r="X67" s="6"/>
-      <c r="Y67" s="6"/>
-      <c r="Z67" s="6"/>
-      <c r="AA67" s="6"/>
-      <c r="AB67" s="6"/>
-      <c r="AC67" s="6"/>
-      <c r="AD67" s="6"/>
-      <c r="AE67" s="6"/>
-      <c r="AF67" s="6"/>
-      <c r="AG67" s="6"/>
-    </row>
-    <row r="69" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B69" s="4" t="s">
+      <c r="C64" s="6"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6"/>
+      <c r="H64" s="6"/>
+      <c r="I64" s="6"/>
+      <c r="J64" s="6"/>
+      <c r="K64" s="6"/>
+      <c r="L64" s="6"/>
+      <c r="M64" s="6"/>
+      <c r="N64" s="6"/>
+      <c r="O64" s="6"/>
+      <c r="P64" s="6"/>
+      <c r="Q64" s="6"/>
+      <c r="R64" s="6"/>
+      <c r="S64" s="6"/>
+      <c r="T64" s="6"/>
+      <c r="U64" s="6"/>
+      <c r="V64" s="6"/>
+      <c r="W64" s="6"/>
+      <c r="X64" s="6"/>
+      <c r="Y64" s="6"/>
+      <c r="Z64" s="6"/>
+      <c r="AA64" s="6"/>
+      <c r="AB64" s="6"/>
+      <c r="AC64" s="6"/>
+      <c r="AD64" s="6"/>
+      <c r="AE64" s="6"/>
+      <c r="AF64" s="6"/>
+      <c r="AG64" s="6"/>
+    </row>
+    <row r="66" ht="21" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B66" s="4" t="s">
         <v>615</v>
       </c>
-      <c r="C69" s="4"/>
-      <c r="D69" s="4"/>
-      <c r="E69" s="4"/>
-      <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
-      <c r="H69" s="4"/>
-      <c r="I69" s="4"/>
-      <c r="J69" s="4"/>
-      <c r="K69" s="4"/>
-      <c r="L69" s="4"/>
-      <c r="M69" s="4"/>
-      <c r="N69" s="4"/>
-      <c r="O69" s="4"/>
-      <c r="P69" s="4"/>
-      <c r="Q69" s="4"/>
-      <c r="R69" s="4"/>
-      <c r="S69" s="4"/>
-      <c r="T69" s="4"/>
-      <c r="U69" s="4"/>
-      <c r="V69" s="4"/>
-      <c r="W69" s="4"/>
-      <c r="X69" s="4"/>
-      <c r="Y69" s="4"/>
-      <c r="Z69" s="4"/>
-      <c r="AA69" s="4"/>
-      <c r="AB69" s="4"/>
-      <c r="AC69" s="4"/>
-      <c r="AD69" s="4"/>
-      <c r="AE69" s="4"/>
-      <c r="AF69" s="4"/>
-      <c r="AG69" s="4"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="4"/>
+      <c r="F66" s="4"/>
+      <c r="G66" s="4"/>
+      <c r="H66" s="4"/>
+      <c r="I66" s="4"/>
+      <c r="J66" s="4"/>
+      <c r="K66" s="4"/>
+      <c r="L66" s="4"/>
+      <c r="M66" s="4"/>
+      <c r="N66" s="4"/>
+      <c r="O66" s="4"/>
+      <c r="P66" s="4"/>
+      <c r="Q66" s="4"/>
+      <c r="R66" s="4"/>
+      <c r="S66" s="4"/>
+      <c r="T66" s="4"/>
+      <c r="U66" s="4"/>
+      <c r="V66" s="4"/>
+      <c r="W66" s="4"/>
+      <c r="X66" s="4"/>
+      <c r="Y66" s="4"/>
+      <c r="Z66" s="4"/>
+      <c r="AA66" s="4"/>
+      <c r="AB66" s="4"/>
+      <c r="AC66" s="4"/>
+      <c r="AD66" s="4"/>
+      <c r="AE66" s="4"/>
+      <c r="AF66" s="4"/>
+      <c r="AG66" s="4"/>
+    </row>
+    <row r="67" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B67" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>616</v>
+      </c>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
+      <c r="H67" s="5"/>
+      <c r="I67" s="5"/>
+      <c r="J67" s="5"/>
+      <c r="K67" s="5"/>
+      <c r="L67" s="5"/>
+      <c r="M67" s="5" t="s">
+        <v>618</v>
+      </c>
+      <c r="N67" s="5"/>
+      <c r="O67" s="5"/>
+      <c r="P67" s="5"/>
+      <c r="Q67" s="5"/>
+      <c r="R67" s="5"/>
+      <c r="S67" s="5"/>
+      <c r="T67" s="5" t="s">
+        <v>619</v>
+      </c>
+      <c r="U67" s="5"/>
+      <c r="V67" s="5"/>
+      <c r="W67" s="5"/>
+      <c r="X67" s="5"/>
+      <c r="Y67" s="5"/>
+      <c r="Z67" s="5"/>
+      <c r="AA67" s="5"/>
+      <c r="AB67" s="5"/>
+      <c r="AC67" s="5"/>
+      <c r="AD67" s="5"/>
+      <c r="AE67" s="5" t="s">
+        <v>620</v>
+      </c>
+      <c r="AF67" s="5"/>
+      <c r="AG67" s="5"/>
+    </row>
+    <row r="68" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B68" s="8">
+        <v>1</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>621</v>
+      </c>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+      <c r="H68" s="3"/>
+      <c r="I68" s="3"/>
+      <c r="J68" s="3"/>
+      <c r="K68" s="3"/>
+      <c r="L68" s="3"/>
+      <c r="M68" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="N68" s="3"/>
+      <c r="O68" s="3"/>
+      <c r="P68" s="3"/>
+      <c r="Q68" s="3"/>
+      <c r="R68" s="3"/>
+      <c r="S68" s="3"/>
+      <c r="T68" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="U68" s="3"/>
+      <c r="V68" s="3"/>
+      <c r="W68" s="3"/>
+      <c r="X68" s="3"/>
+      <c r="Y68" s="3"/>
+      <c r="Z68" s="3"/>
+      <c r="AA68" s="3"/>
+      <c r="AB68" s="3"/>
+      <c r="AC68" s="3"/>
+      <c r="AD68" s="3"/>
+      <c r="AE68" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="AF68" s="3"/>
+      <c r="AG68" s="3"/>
+    </row>
+    <row r="69" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B69" s="8">
+        <v>2</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>621</v>
+      </c>
+      <c r="D69" s="3"/>
+      <c r="E69" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="3"/>
+      <c r="I69" s="3"/>
+      <c r="J69" s="3"/>
+      <c r="K69" s="3"/>
+      <c r="L69" s="3"/>
+      <c r="M69" s="3" t="s">
+        <v>627</v>
+      </c>
+      <c r="N69" s="3"/>
+      <c r="O69" s="3"/>
+      <c r="P69" s="3"/>
+      <c r="Q69" s="3"/>
+      <c r="R69" s="3"/>
+      <c r="S69" s="3"/>
+      <c r="T69" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="U69" s="3"/>
+      <c r="V69" s="3"/>
+      <c r="W69" s="3"/>
+      <c r="X69" s="3"/>
+      <c r="Y69" s="3"/>
+      <c r="Z69" s="3"/>
+      <c r="AA69" s="3"/>
+      <c r="AB69" s="3"/>
+      <c r="AC69" s="3"/>
+      <c r="AD69" s="3"/>
+      <c r="AE69" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="AF69" s="3"/>
+      <c r="AG69" s="3"/>
     </row>
     <row r="70" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B70" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="C70" s="5" t="s">
-        <v>616</v>
-      </c>
-      <c r="D70" s="5"/>
-      <c r="E70" s="5" t="s">
-        <v>617</v>
-      </c>
-      <c r="F70" s="5"/>
-      <c r="G70" s="5"/>
-      <c r="H70" s="5"/>
-      <c r="I70" s="5"/>
-      <c r="J70" s="5"/>
-      <c r="K70" s="5"/>
-      <c r="L70" s="5"/>
-      <c r="M70" s="5" t="s">
-        <v>618</v>
-      </c>
-      <c r="N70" s="5"/>
-      <c r="O70" s="5"/>
-      <c r="P70" s="5"/>
-      <c r="Q70" s="5"/>
-      <c r="R70" s="5"/>
-      <c r="S70" s="5"/>
-      <c r="T70" s="5" t="s">
-        <v>619</v>
-      </c>
-      <c r="U70" s="5"/>
-      <c r="V70" s="5"/>
-      <c r="W70" s="5"/>
-      <c r="X70" s="5"/>
-      <c r="Y70" s="5"/>
-      <c r="Z70" s="5"/>
-      <c r="AA70" s="5"/>
-      <c r="AB70" s="5"/>
-      <c r="AC70" s="5"/>
-      <c r="AD70" s="5"/>
-      <c r="AE70" s="5" t="s">
-        <v>620</v>
-      </c>
-      <c r="AF70" s="5"/>
-      <c r="AG70" s="5"/>
+      <c r="B70" s="8">
+        <v>3</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>621</v>
+      </c>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3" t="s">
+        <v>630</v>
+      </c>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="3"/>
+      <c r="J70" s="3"/>
+      <c r="K70" s="3"/>
+      <c r="L70" s="3"/>
+      <c r="M70" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="N70" s="3"/>
+      <c r="O70" s="3"/>
+      <c r="P70" s="3"/>
+      <c r="Q70" s="3"/>
+      <c r="R70" s="3"/>
+      <c r="S70" s="3"/>
+      <c r="T70" s="3" t="s">
+        <v>631</v>
+      </c>
+      <c r="U70" s="3"/>
+      <c r="V70" s="3"/>
+      <c r="W70" s="3"/>
+      <c r="X70" s="3"/>
+      <c r="Y70" s="3"/>
+      <c r="Z70" s="3"/>
+      <c r="AA70" s="3"/>
+      <c r="AB70" s="3"/>
+      <c r="AC70" s="3"/>
+      <c r="AD70" s="3"/>
+      <c r="AE70" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="AF70" s="3"/>
+      <c r="AG70" s="3"/>
     </row>
     <row r="71" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B71" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D71" s="3"/>
       <c r="E71" s="3" t="s">
-        <v>622</v>
+        <v>633</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -20954,7 +21092,7 @@
       <c r="K71" s="3"/>
       <c r="L71" s="3"/>
       <c r="M71" s="3" t="s">
-        <v>623</v>
+        <v>634</v>
       </c>
       <c r="N71" s="3"/>
       <c r="O71" s="3"/>
@@ -20963,7 +21101,7 @@
       <c r="R71" s="3"/>
       <c r="S71" s="3"/>
       <c r="T71" s="3" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="U71" s="3"/>
       <c r="V71" s="3"/>
@@ -20976,21 +21114,21 @@
       <c r="AC71" s="3"/>
       <c r="AD71" s="3"/>
       <c r="AE71" s="3" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
       <c r="AF71" s="3"/>
       <c r="AG71" s="3"/>
     </row>
-    <row r="72" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B72" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>621</v>
       </c>
       <c r="D72" s="3"/>
       <c r="E72" s="3" t="s">
-        <v>626</v>
+        <v>637</v>
       </c>
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
@@ -21000,7 +21138,7 @@
       <c r="K72" s="3"/>
       <c r="L72" s="3"/>
       <c r="M72" s="3" t="s">
-        <v>627</v>
+        <v>634</v>
       </c>
       <c r="N72" s="3"/>
       <c r="O72" s="3"/>
@@ -21009,7 +21147,7 @@
       <c r="R72" s="3"/>
       <c r="S72" s="3"/>
       <c r="T72" s="3" t="s">
-        <v>628</v>
+        <v>638</v>
       </c>
       <c r="U72" s="3"/>
       <c r="V72" s="3"/>
@@ -21022,21 +21160,21 @@
       <c r="AC72" s="3"/>
       <c r="AD72" s="3"/>
       <c r="AE72" s="3" t="s">
-        <v>629</v>
+        <v>639</v>
       </c>
       <c r="AF72" s="3"/>
       <c r="AG72" s="3"/>
     </row>
-    <row r="73" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="73" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B73" s="8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D73" s="3"/>
       <c r="E73" s="3" t="s">
-        <v>630</v>
+        <v>640</v>
       </c>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
@@ -21046,7 +21184,7 @@
       <c r="K73" s="3"/>
       <c r="L73" s="3"/>
       <c r="M73" s="3" t="s">
-        <v>623</v>
+        <v>641</v>
       </c>
       <c r="N73" s="3"/>
       <c r="O73" s="3"/>
@@ -21055,7 +21193,7 @@
       <c r="R73" s="3"/>
       <c r="S73" s="3"/>
       <c r="T73" s="3" t="s">
-        <v>631</v>
+        <v>642</v>
       </c>
       <c r="U73" s="3"/>
       <c r="V73" s="3"/>
@@ -21068,21 +21206,21 @@
       <c r="AC73" s="3"/>
       <c r="AD73" s="3"/>
       <c r="AE73" s="3" t="s">
-        <v>629</v>
+        <v>643</v>
       </c>
       <c r="AF73" s="3"/>
       <c r="AG73" s="3"/>
     </row>
     <row r="74" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B74" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>632</v>
       </c>
       <c r="D74" s="3"/>
       <c r="E74" s="3" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
       <c r="F74" s="3"/>
       <c r="G74" s="3"/>
@@ -21092,7 +21230,7 @@
       <c r="K74" s="3"/>
       <c r="L74" s="3"/>
       <c r="M74" s="3" t="s">
-        <v>634</v>
+        <v>645</v>
       </c>
       <c r="N74" s="3"/>
       <c r="O74" s="3"/>
@@ -21101,7 +21239,7 @@
       <c r="R74" s="3"/>
       <c r="S74" s="3"/>
       <c r="T74" s="3" t="s">
-        <v>635</v>
+        <v>646</v>
       </c>
       <c r="U74" s="3"/>
       <c r="V74" s="3"/>
@@ -21114,21 +21252,21 @@
       <c r="AC74" s="3"/>
       <c r="AD74" s="3"/>
       <c r="AE74" s="3" t="s">
-        <v>636</v>
+        <v>629</v>
       </c>
       <c r="AF74" s="3"/>
       <c r="AG74" s="3"/>
     </row>
-    <row r="75" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="75" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B75" s="8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D75" s="3"/>
       <c r="E75" s="3" t="s">
-        <v>637</v>
+        <v>647</v>
       </c>
       <c r="F75" s="3"/>
       <c r="G75" s="3"/>
@@ -21138,7 +21276,7 @@
       <c r="K75" s="3"/>
       <c r="L75" s="3"/>
       <c r="M75" s="3" t="s">
-        <v>634</v>
+        <v>648</v>
       </c>
       <c r="N75" s="3"/>
       <c r="O75" s="3"/>
@@ -21147,7 +21285,7 @@
       <c r="R75" s="3"/>
       <c r="S75" s="3"/>
       <c r="T75" s="3" t="s">
-        <v>638</v>
+        <v>649</v>
       </c>
       <c r="U75" s="3"/>
       <c r="V75" s="3"/>
@@ -21160,21 +21298,21 @@
       <c r="AC75" s="3"/>
       <c r="AD75" s="3"/>
       <c r="AE75" s="3" t="s">
-        <v>639</v>
+        <v>650</v>
       </c>
       <c r="AF75" s="3"/>
       <c r="AG75" s="3"/>
     </row>
     <row r="76" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B76" s="8">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C76" s="3" t="s">
         <v>632</v>
       </c>
       <c r="D76" s="3"/>
       <c r="E76" s="3" t="s">
-        <v>640</v>
+        <v>651</v>
       </c>
       <c r="F76" s="3"/>
       <c r="G76" s="3"/>
@@ -21184,7 +21322,7 @@
       <c r="K76" s="3"/>
       <c r="L76" s="3"/>
       <c r="M76" s="3" t="s">
-        <v>641</v>
+        <v>648</v>
       </c>
       <c r="N76" s="3"/>
       <c r="O76" s="3"/>
@@ -21193,7 +21331,7 @@
       <c r="R76" s="3"/>
       <c r="S76" s="3"/>
       <c r="T76" s="3" t="s">
-        <v>642</v>
+        <v>652</v>
       </c>
       <c r="U76" s="3"/>
       <c r="V76" s="3"/>
@@ -21206,21 +21344,21 @@
       <c r="AC76" s="3"/>
       <c r="AD76" s="3"/>
       <c r="AE76" s="3" t="s">
-        <v>643</v>
+        <v>653</v>
       </c>
       <c r="AF76" s="3"/>
       <c r="AG76" s="3"/>
     </row>
-    <row r="77" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B77" s="8">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C77" s="3" t="s">
         <v>632</v>
       </c>
       <c r="D77" s="3"/>
       <c r="E77" s="3" t="s">
-        <v>644</v>
+        <v>654</v>
       </c>
       <c r="F77" s="3"/>
       <c r="G77" s="3"/>
@@ -21230,7 +21368,7 @@
       <c r="K77" s="3"/>
       <c r="L77" s="3"/>
       <c r="M77" s="3" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="N77" s="3"/>
       <c r="O77" s="3"/>
@@ -21239,7 +21377,7 @@
       <c r="R77" s="3"/>
       <c r="S77" s="3"/>
       <c r="T77" s="3" t="s">
-        <v>646</v>
+        <v>655</v>
       </c>
       <c r="U77" s="3"/>
       <c r="V77" s="3"/>
@@ -21252,21 +21390,21 @@
       <c r="AC77" s="3"/>
       <c r="AD77" s="3"/>
       <c r="AE77" s="3" t="s">
-        <v>629</v>
+        <v>656</v>
       </c>
       <c r="AF77" s="3"/>
       <c r="AG77" s="3"/>
     </row>
-    <row r="78" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="78" ht="43" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B78" s="8">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>632</v>
       </c>
       <c r="D78" s="3"/>
       <c r="E78" s="3" t="s">
-        <v>647</v>
+        <v>657</v>
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="3"/>
@@ -21276,7 +21414,7 @@
       <c r="K78" s="3"/>
       <c r="L78" s="3"/>
       <c r="M78" s="3" t="s">
-        <v>648</v>
+        <v>658</v>
       </c>
       <c r="N78" s="3"/>
       <c r="O78" s="3"/>
@@ -21285,7 +21423,7 @@
       <c r="R78" s="3"/>
       <c r="S78" s="3"/>
       <c r="T78" s="3" t="s">
-        <v>649</v>
+        <v>659</v>
       </c>
       <c r="U78" s="3"/>
       <c r="V78" s="3"/>
@@ -21298,21 +21436,21 @@
       <c r="AC78" s="3"/>
       <c r="AD78" s="3"/>
       <c r="AE78" s="3" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="AF78" s="3"/>
       <c r="AG78" s="3"/>
     </row>
     <row r="79" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B79" s="8">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>632</v>
+        <v>621</v>
       </c>
       <c r="D79" s="3"/>
       <c r="E79" s="3" t="s">
-        <v>651</v>
+        <v>660</v>
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
@@ -21331,7 +21469,7 @@
       <c r="R79" s="3"/>
       <c r="S79" s="3"/>
       <c r="T79" s="3" t="s">
-        <v>652</v>
+        <v>661</v>
       </c>
       <c r="U79" s="3"/>
       <c r="V79" s="3"/>
@@ -21344,21 +21482,21 @@
       <c r="AC79" s="3"/>
       <c r="AD79" s="3"/>
       <c r="AE79" s="3" t="s">
-        <v>653</v>
+        <v>662</v>
       </c>
       <c r="AF79" s="3"/>
       <c r="AG79" s="3"/>
     </row>
     <row r="80" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B80" s="8">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>632</v>
+        <v>621</v>
       </c>
       <c r="D80" s="3"/>
       <c r="E80" s="3" t="s">
-        <v>654</v>
+        <v>647</v>
       </c>
       <c r="F80" s="3"/>
       <c r="G80" s="3"/>
@@ -21377,7 +21515,7 @@
       <c r="R80" s="3"/>
       <c r="S80" s="3"/>
       <c r="T80" s="3" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
       <c r="U80" s="3"/>
       <c r="V80" s="3"/>
@@ -21390,21 +21528,21 @@
       <c r="AC80" s="3"/>
       <c r="AD80" s="3"/>
       <c r="AE80" s="3" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="AF80" s="3"/>
       <c r="AG80" s="3"/>
     </row>
-    <row r="81" ht="43" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B81" s="8">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>632</v>
+        <v>664</v>
       </c>
       <c r="D81" s="3"/>
       <c r="E81" s="3" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="F81" s="3"/>
       <c r="G81" s="3"/>
@@ -21414,7 +21552,7 @@
       <c r="K81" s="3"/>
       <c r="L81" s="3"/>
       <c r="M81" s="3" t="s">
-        <v>658</v>
+        <v>665</v>
       </c>
       <c r="N81" s="3"/>
       <c r="O81" s="3"/>
@@ -21423,7 +21561,7 @@
       <c r="R81" s="3"/>
       <c r="S81" s="3"/>
       <c r="T81" s="3" t="s">
-        <v>659</v>
+        <v>666</v>
       </c>
       <c r="U81" s="3"/>
       <c r="V81" s="3"/>
@@ -21436,21 +21574,21 @@
       <c r="AC81" s="3"/>
       <c r="AD81" s="3"/>
       <c r="AE81" s="3" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="AF81" s="3"/>
       <c r="AG81" s="3"/>
     </row>
-    <row r="82" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B82" s="8">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>621</v>
       </c>
       <c r="D82" s="3"/>
       <c r="E82" s="3" t="s">
-        <v>660</v>
+        <v>667</v>
       </c>
       <c r="F82" s="3"/>
       <c r="G82" s="3"/>
@@ -21469,7 +21607,7 @@
       <c r="R82" s="3"/>
       <c r="S82" s="3"/>
       <c r="T82" s="3" t="s">
-        <v>661</v>
+        <v>668</v>
       </c>
       <c r="U82" s="3"/>
       <c r="V82" s="3"/>
@@ -21482,21 +21620,21 @@
       <c r="AC82" s="3"/>
       <c r="AD82" s="3"/>
       <c r="AE82" s="3" t="s">
-        <v>662</v>
+        <v>656</v>
       </c>
       <c r="AF82" s="3"/>
       <c r="AG82" s="3"/>
     </row>
     <row r="83" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B83" s="8">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C83" s="3" t="s">
         <v>621</v>
       </c>
       <c r="D83" s="3"/>
       <c r="E83" s="3" t="s">
-        <v>647</v>
+        <v>669</v>
       </c>
       <c r="F83" s="3"/>
       <c r="G83" s="3"/>
@@ -21515,7 +21653,7 @@
       <c r="R83" s="3"/>
       <c r="S83" s="3"/>
       <c r="T83" s="3" t="s">
-        <v>663</v>
+        <v>670</v>
       </c>
       <c r="U83" s="3"/>
       <c r="V83" s="3"/>
@@ -21528,21 +21666,21 @@
       <c r="AC83" s="3"/>
       <c r="AD83" s="3"/>
       <c r="AE83" s="3" t="s">
-        <v>662</v>
+        <v>656</v>
       </c>
       <c r="AF83" s="3"/>
       <c r="AG83" s="3"/>
     </row>
     <row r="84" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B84" s="8">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>664</v>
+        <v>621</v>
       </c>
       <c r="D84" s="3"/>
       <c r="E84" s="3" t="s">
-        <v>654</v>
+        <v>671</v>
       </c>
       <c r="F84" s="3"/>
       <c r="G84" s="3"/>
@@ -21552,7 +21690,7 @@
       <c r="K84" s="3"/>
       <c r="L84" s="3"/>
       <c r="M84" s="3" t="s">
-        <v>665</v>
+        <v>648</v>
       </c>
       <c r="N84" s="3"/>
       <c r="O84" s="3"/>
@@ -21561,7 +21699,7 @@
       <c r="R84" s="3"/>
       <c r="S84" s="3"/>
       <c r="T84" s="3" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="U84" s="3"/>
       <c r="V84" s="3"/>
@@ -21574,21 +21712,21 @@
       <c r="AC84" s="3"/>
       <c r="AD84" s="3"/>
       <c r="AE84" s="3" t="s">
-        <v>662</v>
+        <v>656</v>
       </c>
       <c r="AF84" s="3"/>
       <c r="AG84" s="3"/>
     </row>
     <row r="85" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B85" s="8">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>621</v>
       </c>
       <c r="D85" s="3"/>
       <c r="E85" s="3" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="F85" s="3"/>
       <c r="G85" s="3"/>
@@ -21607,7 +21745,7 @@
       <c r="R85" s="3"/>
       <c r="S85" s="3"/>
       <c r="T85" s="3" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="U85" s="3"/>
       <c r="V85" s="3"/>
@@ -21620,21 +21758,21 @@
       <c r="AC85" s="3"/>
       <c r="AD85" s="3"/>
       <c r="AE85" s="3" t="s">
-        <v>656</v>
+        <v>675</v>
       </c>
       <c r="AF85" s="3"/>
       <c r="AG85" s="3"/>
     </row>
     <row r="86" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B86" s="8">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>621</v>
       </c>
       <c r="D86" s="3"/>
       <c r="E86" s="3" t="s">
-        <v>669</v>
+        <v>676</v>
       </c>
       <c r="F86" s="3"/>
       <c r="G86" s="3"/>
@@ -21653,7 +21791,7 @@
       <c r="R86" s="3"/>
       <c r="S86" s="3"/>
       <c r="T86" s="3" t="s">
-        <v>670</v>
+        <v>677</v>
       </c>
       <c r="U86" s="3"/>
       <c r="V86" s="3"/>
@@ -21666,21 +21804,21 @@
       <c r="AC86" s="3"/>
       <c r="AD86" s="3"/>
       <c r="AE86" s="3" t="s">
-        <v>656</v>
+        <v>675</v>
       </c>
       <c r="AF86" s="3"/>
       <c r="AG86" s="3"/>
     </row>
     <row r="87" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B87" s="8">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D87" s="3"/>
       <c r="E87" s="3" t="s">
-        <v>671</v>
+        <v>678</v>
       </c>
       <c r="F87" s="3"/>
       <c r="G87" s="3"/>
@@ -21699,7 +21837,7 @@
       <c r="R87" s="3"/>
       <c r="S87" s="3"/>
       <c r="T87" s="3" t="s">
-        <v>672</v>
+        <v>679</v>
       </c>
       <c r="U87" s="3"/>
       <c r="V87" s="3"/>
@@ -21717,16 +21855,16 @@
       <c r="AF87" s="3"/>
       <c r="AG87" s="3"/>
     </row>
-    <row r="88" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="88" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B88" s="8">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C88" s="3" t="s">
         <v>621</v>
       </c>
       <c r="D88" s="3"/>
       <c r="E88" s="3" t="s">
-        <v>673</v>
+        <v>680</v>
       </c>
       <c r="F88" s="3"/>
       <c r="G88" s="3"/>
@@ -21736,7 +21874,7 @@
       <c r="K88" s="3"/>
       <c r="L88" s="3"/>
       <c r="M88" s="3" t="s">
-        <v>648</v>
+        <v>681</v>
       </c>
       <c r="N88" s="3"/>
       <c r="O88" s="3"/>
@@ -21745,7 +21883,7 @@
       <c r="R88" s="3"/>
       <c r="S88" s="3"/>
       <c r="T88" s="3" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="U88" s="3"/>
       <c r="V88" s="3"/>
@@ -21758,21 +21896,21 @@
       <c r="AC88" s="3"/>
       <c r="AD88" s="3"/>
       <c r="AE88" s="3" t="s">
-        <v>675</v>
+        <v>656</v>
       </c>
       <c r="AF88" s="3"/>
       <c r="AG88" s="3"/>
     </row>
     <row r="89" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B89" s="8">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>621</v>
       </c>
       <c r="D89" s="3"/>
       <c r="E89" s="3" t="s">
-        <v>676</v>
+        <v>683</v>
       </c>
       <c r="F89" s="3"/>
       <c r="G89" s="3"/>
@@ -21791,7 +21929,7 @@
       <c r="R89" s="3"/>
       <c r="S89" s="3"/>
       <c r="T89" s="3" t="s">
-        <v>677</v>
+        <v>684</v>
       </c>
       <c r="U89" s="3"/>
       <c r="V89" s="3"/>
@@ -21804,21 +21942,21 @@
       <c r="AC89" s="3"/>
       <c r="AD89" s="3"/>
       <c r="AE89" s="3" t="s">
-        <v>675</v>
+        <v>656</v>
       </c>
       <c r="AF89" s="3"/>
       <c r="AG89" s="3"/>
     </row>
     <row r="90" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B90" s="8">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>632</v>
+        <v>664</v>
       </c>
       <c r="D90" s="3"/>
       <c r="E90" s="3" t="s">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="F90" s="3"/>
       <c r="G90" s="3"/>
@@ -21828,7 +21966,7 @@
       <c r="K90" s="3"/>
       <c r="L90" s="3"/>
       <c r="M90" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N90" s="3"/>
       <c r="O90" s="3"/>
@@ -21837,7 +21975,7 @@
       <c r="R90" s="3"/>
       <c r="S90" s="3"/>
       <c r="T90" s="3" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="U90" s="3"/>
       <c r="V90" s="3"/>
@@ -21855,16 +21993,16 @@
       <c r="AF90" s="3"/>
       <c r="AG90" s="3"/>
     </row>
-    <row r="91" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B91" s="8">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>621</v>
+        <v>688</v>
       </c>
       <c r="D91" s="3"/>
       <c r="E91" s="3" t="s">
-        <v>680</v>
+        <v>685</v>
       </c>
       <c r="F91" s="3"/>
       <c r="G91" s="3"/>
@@ -21874,7 +22012,7 @@
       <c r="K91" s="3"/>
       <c r="L91" s="3"/>
       <c r="M91" s="3" t="s">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="N91" s="3"/>
       <c r="O91" s="3"/>
@@ -21883,7 +22021,7 @@
       <c r="R91" s="3"/>
       <c r="S91" s="3"/>
       <c r="T91" s="3" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
       <c r="U91" s="3"/>
       <c r="V91" s="3"/>
@@ -21903,14 +22041,14 @@
     </row>
     <row r="92" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B92" s="8">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D92" s="3"/>
       <c r="E92" s="3" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="F92" s="3"/>
       <c r="G92" s="3"/>
@@ -21929,7 +22067,7 @@
       <c r="R92" s="3"/>
       <c r="S92" s="3"/>
       <c r="T92" s="3" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="U92" s="3"/>
       <c r="V92" s="3"/>
@@ -21942,21 +22080,21 @@
       <c r="AC92" s="3"/>
       <c r="AD92" s="3"/>
       <c r="AE92" s="3" t="s">
-        <v>656</v>
+        <v>692</v>
       </c>
       <c r="AF92" s="3"/>
       <c r="AG92" s="3"/>
     </row>
     <row r="93" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B93" s="8">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>664</v>
+        <v>632</v>
       </c>
       <c r="D93" s="3"/>
       <c r="E93" s="3" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="F93" s="3"/>
       <c r="G93" s="3"/>
@@ -21966,7 +22104,7 @@
       <c r="K93" s="3"/>
       <c r="L93" s="3"/>
       <c r="M93" s="3" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
       <c r="N93" s="3"/>
       <c r="O93" s="3"/>
@@ -21975,7 +22113,7 @@
       <c r="R93" s="3"/>
       <c r="S93" s="3"/>
       <c r="T93" s="3" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="U93" s="3"/>
       <c r="V93" s="3"/>
@@ -21988,21 +22126,21 @@
       <c r="AC93" s="3"/>
       <c r="AD93" s="3"/>
       <c r="AE93" s="3" t="s">
-        <v>656</v>
+        <v>695</v>
       </c>
       <c r="AF93" s="3"/>
       <c r="AG93" s="3"/>
     </row>
     <row r="94" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B94" s="8">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>688</v>
+        <v>621</v>
       </c>
       <c r="D94" s="3"/>
       <c r="E94" s="3" t="s">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="F94" s="3"/>
       <c r="G94" s="3"/>
@@ -22021,7 +22159,7 @@
       <c r="R94" s="3"/>
       <c r="S94" s="3"/>
       <c r="T94" s="3" t="s">
-        <v>689</v>
+        <v>696</v>
       </c>
       <c r="U94" s="3"/>
       <c r="V94" s="3"/>
@@ -22034,21 +22172,21 @@
       <c r="AC94" s="3"/>
       <c r="AD94" s="3"/>
       <c r="AE94" s="3" t="s">
-        <v>656</v>
+        <v>697</v>
       </c>
       <c r="AF94" s="3"/>
       <c r="AG94" s="3"/>
     </row>
     <row r="95" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B95" s="8">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>632</v>
+        <v>664</v>
       </c>
       <c r="D95" s="3"/>
       <c r="E95" s="3" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="F95" s="3"/>
       <c r="G95" s="3"/>
@@ -22058,7 +22196,7 @@
       <c r="K95" s="3"/>
       <c r="L95" s="3"/>
       <c r="M95" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N95" s="3"/>
       <c r="O95" s="3"/>
@@ -22067,7 +22205,7 @@
       <c r="R95" s="3"/>
       <c r="S95" s="3"/>
       <c r="T95" s="3" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
       <c r="U95" s="3"/>
       <c r="V95" s="3"/>
@@ -22080,21 +22218,21 @@
       <c r="AC95" s="3"/>
       <c r="AD95" s="3"/>
       <c r="AE95" s="3" t="s">
-        <v>692</v>
+        <v>697</v>
       </c>
       <c r="AF95" s="3"/>
       <c r="AG95" s="3"/>
     </row>
     <row r="96" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B96" s="8">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>632</v>
+        <v>699</v>
       </c>
       <c r="D96" s="3"/>
       <c r="E96" s="3" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="F96" s="3"/>
       <c r="G96" s="3"/>
@@ -22104,7 +22242,7 @@
       <c r="K96" s="3"/>
       <c r="L96" s="3"/>
       <c r="M96" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N96" s="3"/>
       <c r="O96" s="3"/>
@@ -22113,7 +22251,7 @@
       <c r="R96" s="3"/>
       <c r="S96" s="3"/>
       <c r="T96" s="3" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
       <c r="U96" s="3"/>
       <c r="V96" s="3"/>
@@ -22126,21 +22264,21 @@
       <c r="AC96" s="3"/>
       <c r="AD96" s="3"/>
       <c r="AE96" s="3" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
       <c r="AF96" s="3"/>
       <c r="AG96" s="3"/>
     </row>
     <row r="97" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B97" s="8">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C97" s="3" t="s">
         <v>621</v>
       </c>
       <c r="D97" s="3"/>
       <c r="E97" s="3" t="s">
-        <v>690</v>
+        <v>703</v>
       </c>
       <c r="F97" s="3"/>
       <c r="G97" s="3"/>
@@ -22150,7 +22288,7 @@
       <c r="K97" s="3"/>
       <c r="L97" s="3"/>
       <c r="M97" s="3" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
       <c r="N97" s="3"/>
       <c r="O97" s="3"/>
@@ -22159,7 +22297,7 @@
       <c r="R97" s="3"/>
       <c r="S97" s="3"/>
       <c r="T97" s="3" t="s">
-        <v>696</v>
+        <v>704</v>
       </c>
       <c r="U97" s="3"/>
       <c r="V97" s="3"/>
@@ -22172,21 +22310,21 @@
       <c r="AC97" s="3"/>
       <c r="AD97" s="3"/>
       <c r="AE97" s="3" t="s">
-        <v>697</v>
+        <v>705</v>
       </c>
       <c r="AF97" s="3"/>
       <c r="AG97" s="3"/>
     </row>
     <row r="98" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B98" s="8">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>664</v>
+        <v>621</v>
       </c>
       <c r="D98" s="3"/>
       <c r="E98" s="3" t="s">
-        <v>693</v>
+        <v>706</v>
       </c>
       <c r="F98" s="3"/>
       <c r="G98" s="3"/>
@@ -22205,7 +22343,7 @@
       <c r="R98" s="3"/>
       <c r="S98" s="3"/>
       <c r="T98" s="3" t="s">
-        <v>698</v>
+        <v>707</v>
       </c>
       <c r="U98" s="3"/>
       <c r="V98" s="3"/>
@@ -22225,14 +22363,14 @@
     </row>
     <row r="99" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B99" s="8">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>699</v>
+        <v>688</v>
       </c>
       <c r="D99" s="3"/>
       <c r="E99" s="3" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="F99" s="3"/>
       <c r="G99" s="3"/>
@@ -22251,7 +22389,7 @@
       <c r="R99" s="3"/>
       <c r="S99" s="3"/>
       <c r="T99" s="3" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="U99" s="3"/>
       <c r="V99" s="3"/>
@@ -22264,21 +22402,21 @@
       <c r="AC99" s="3"/>
       <c r="AD99" s="3"/>
       <c r="AE99" s="3" t="s">
-        <v>702</v>
+        <v>697</v>
       </c>
       <c r="AF99" s="3"/>
       <c r="AG99" s="3"/>
     </row>
     <row r="100" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B100" s="8">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D100" s="3"/>
       <c r="E100" s="3" t="s">
-        <v>703</v>
+        <v>710</v>
       </c>
       <c r="F100" s="3"/>
       <c r="G100" s="3"/>
@@ -22297,7 +22435,7 @@
       <c r="R100" s="3"/>
       <c r="S100" s="3"/>
       <c r="T100" s="3" t="s">
-        <v>704</v>
+        <v>711</v>
       </c>
       <c r="U100" s="3"/>
       <c r="V100" s="3"/>
@@ -22310,21 +22448,21 @@
       <c r="AC100" s="3"/>
       <c r="AD100" s="3"/>
       <c r="AE100" s="3" t="s">
-        <v>705</v>
+        <v>712</v>
       </c>
       <c r="AF100" s="3"/>
       <c r="AG100" s="3"/>
     </row>
-    <row r="101" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="101" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B101" s="8">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D101" s="3"/>
       <c r="E101" s="3" t="s">
-        <v>706</v>
+        <v>713</v>
       </c>
       <c r="F101" s="3"/>
       <c r="G101" s="3"/>
@@ -22334,7 +22472,7 @@
       <c r="K101" s="3"/>
       <c r="L101" s="3"/>
       <c r="M101" s="3" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
       <c r="N101" s="3"/>
       <c r="O101" s="3"/>
@@ -22343,7 +22481,7 @@
       <c r="R101" s="3"/>
       <c r="S101" s="3"/>
       <c r="T101" s="3" t="s">
-        <v>707</v>
+        <v>714</v>
       </c>
       <c r="U101" s="3"/>
       <c r="V101" s="3"/>
@@ -22356,21 +22494,21 @@
       <c r="AC101" s="3"/>
       <c r="AD101" s="3"/>
       <c r="AE101" s="3" t="s">
-        <v>697</v>
+        <v>715</v>
       </c>
       <c r="AF101" s="3"/>
       <c r="AG101" s="3"/>
     </row>
     <row r="102" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B102" s="8">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>688</v>
+        <v>664</v>
       </c>
       <c r="D102" s="3"/>
       <c r="E102" s="3" t="s">
-        <v>708</v>
+        <v>713</v>
       </c>
       <c r="F102" s="3"/>
       <c r="G102" s="3"/>
@@ -22389,7 +22527,7 @@
       <c r="R102" s="3"/>
       <c r="S102" s="3"/>
       <c r="T102" s="3" t="s">
-        <v>709</v>
+        <v>716</v>
       </c>
       <c r="U102" s="3"/>
       <c r="V102" s="3"/>
@@ -22402,21 +22540,21 @@
       <c r="AC102" s="3"/>
       <c r="AD102" s="3"/>
       <c r="AE102" s="3" t="s">
-        <v>697</v>
+        <v>717</v>
       </c>
       <c r="AF102" s="3"/>
       <c r="AG102" s="3"/>
     </row>
     <row r="103" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B103" s="8">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C103" s="3" t="s">
         <v>632</v>
       </c>
       <c r="D103" s="3"/>
       <c r="E103" s="3" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="F103" s="3"/>
       <c r="G103" s="3"/>
@@ -22435,7 +22573,7 @@
       <c r="R103" s="3"/>
       <c r="S103" s="3"/>
       <c r="T103" s="3" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="U103" s="3"/>
       <c r="V103" s="3"/>
@@ -22448,21 +22586,21 @@
       <c r="AC103" s="3"/>
       <c r="AD103" s="3"/>
       <c r="AE103" s="3" t="s">
-        <v>712</v>
+        <v>702</v>
       </c>
       <c r="AF103" s="3"/>
       <c r="AG103" s="3"/>
     </row>
-    <row r="104" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B104" s="8">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>632</v>
+        <v>621</v>
       </c>
       <c r="D104" s="3"/>
       <c r="E104" s="3" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="F104" s="3"/>
       <c r="G104" s="3"/>
@@ -22472,7 +22610,7 @@
       <c r="K104" s="3"/>
       <c r="L104" s="3"/>
       <c r="M104" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N104" s="3"/>
       <c r="O104" s="3"/>
@@ -22481,7 +22619,7 @@
       <c r="R104" s="3"/>
       <c r="S104" s="3"/>
       <c r="T104" s="3" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="U104" s="3"/>
       <c r="V104" s="3"/>
@@ -22494,21 +22632,21 @@
       <c r="AC104" s="3"/>
       <c r="AD104" s="3"/>
       <c r="AE104" s="3" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="AF104" s="3"/>
       <c r="AG104" s="3"/>
     </row>
     <row r="105" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B105" s="8">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C105" s="3" t="s">
         <v>664</v>
       </c>
       <c r="D105" s="3"/>
       <c r="E105" s="3" t="s">
-        <v>713</v>
+        <v>722</v>
       </c>
       <c r="F105" s="3"/>
       <c r="G105" s="3"/>
@@ -22527,7 +22665,7 @@
       <c r="R105" s="3"/>
       <c r="S105" s="3"/>
       <c r="T105" s="3" t="s">
-        <v>716</v>
+        <v>723</v>
       </c>
       <c r="U105" s="3"/>
       <c r="V105" s="3"/>
@@ -22540,21 +22678,21 @@
       <c r="AC105" s="3"/>
       <c r="AD105" s="3"/>
       <c r="AE105" s="3" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="AF105" s="3"/>
       <c r="AG105" s="3"/>
     </row>
     <row r="106" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B106" s="8">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>632</v>
+        <v>699</v>
       </c>
       <c r="D106" s="3"/>
       <c r="E106" s="3" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="F106" s="3"/>
       <c r="G106" s="3"/>
@@ -22564,7 +22702,7 @@
       <c r="K106" s="3"/>
       <c r="L106" s="3"/>
       <c r="M106" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N106" s="3"/>
       <c r="O106" s="3"/>
@@ -22573,7 +22711,7 @@
       <c r="R106" s="3"/>
       <c r="S106" s="3"/>
       <c r="T106" s="3" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="U106" s="3"/>
       <c r="V106" s="3"/>
@@ -22593,14 +22731,14 @@
     </row>
     <row r="107" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B107" s="8">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D107" s="3"/>
       <c r="E107" s="3" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
       <c r="F107" s="3"/>
       <c r="G107" s="3"/>
@@ -22610,7 +22748,7 @@
       <c r="K107" s="3"/>
       <c r="L107" s="3"/>
       <c r="M107" s="3" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
       <c r="N107" s="3"/>
       <c r="O107" s="3"/>
@@ -22619,7 +22757,7 @@
       <c r="R107" s="3"/>
       <c r="S107" s="3"/>
       <c r="T107" s="3" t="s">
-        <v>720</v>
+        <v>727</v>
       </c>
       <c r="U107" s="3"/>
       <c r="V107" s="3"/>
@@ -22632,21 +22770,21 @@
       <c r="AC107" s="3"/>
       <c r="AD107" s="3"/>
       <c r="AE107" s="3" t="s">
-        <v>721</v>
+        <v>728</v>
       </c>
       <c r="AF107" s="3"/>
       <c r="AG107" s="3"/>
     </row>
     <row r="108" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B108" s="8">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>664</v>
+        <v>632</v>
       </c>
       <c r="D108" s="3"/>
       <c r="E108" s="3" t="s">
-        <v>722</v>
+        <v>729</v>
       </c>
       <c r="F108" s="3"/>
       <c r="G108" s="3"/>
@@ -22656,7 +22794,7 @@
       <c r="K108" s="3"/>
       <c r="L108" s="3"/>
       <c r="M108" s="3" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
       <c r="N108" s="3"/>
       <c r="O108" s="3"/>
@@ -22665,7 +22803,7 @@
       <c r="R108" s="3"/>
       <c r="S108" s="3"/>
       <c r="T108" s="3" t="s">
-        <v>723</v>
+        <v>730</v>
       </c>
       <c r="U108" s="3"/>
       <c r="V108" s="3"/>
@@ -22678,21 +22816,21 @@
       <c r="AC108" s="3"/>
       <c r="AD108" s="3"/>
       <c r="AE108" s="3" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="AF108" s="3"/>
       <c r="AG108" s="3"/>
     </row>
     <row r="109" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B109" s="8">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>699</v>
+        <v>621</v>
       </c>
       <c r="D109" s="3"/>
       <c r="E109" s="3" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="F109" s="3"/>
       <c r="G109" s="3"/>
@@ -22711,7 +22849,7 @@
       <c r="R109" s="3"/>
       <c r="S109" s="3"/>
       <c r="T109" s="3" t="s">
-        <v>725</v>
+        <v>732</v>
       </c>
       <c r="U109" s="3"/>
       <c r="V109" s="3"/>
@@ -22724,21 +22862,21 @@
       <c r="AC109" s="3"/>
       <c r="AD109" s="3"/>
       <c r="AE109" s="3" t="s">
-        <v>702</v>
+        <v>731</v>
       </c>
       <c r="AF109" s="3"/>
       <c r="AG109" s="3"/>
     </row>
     <row r="110" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B110" s="8">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>632</v>
+        <v>664</v>
       </c>
       <c r="D110" s="3"/>
       <c r="E110" s="3" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="F110" s="3"/>
       <c r="G110" s="3"/>
@@ -22748,7 +22886,7 @@
       <c r="K110" s="3"/>
       <c r="L110" s="3"/>
       <c r="M110" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N110" s="3"/>
       <c r="O110" s="3"/>
@@ -22757,7 +22895,7 @@
       <c r="R110" s="3"/>
       <c r="S110" s="3"/>
       <c r="T110" s="3" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="U110" s="3"/>
       <c r="V110" s="3"/>
@@ -22770,21 +22908,21 @@
       <c r="AC110" s="3"/>
       <c r="AD110" s="3"/>
       <c r="AE110" s="3" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="AF110" s="3"/>
       <c r="AG110" s="3"/>
     </row>
-    <row r="111" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="111" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B111" s="8">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C111" s="3" t="s">
         <v>632</v>
       </c>
       <c r="D111" s="3"/>
       <c r="E111" s="3" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
       <c r="F111" s="3"/>
       <c r="G111" s="3"/>
@@ -22794,7 +22932,7 @@
       <c r="K111" s="3"/>
       <c r="L111" s="3"/>
       <c r="M111" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N111" s="3"/>
       <c r="O111" s="3"/>
@@ -22803,7 +22941,7 @@
       <c r="R111" s="3"/>
       <c r="S111" s="3"/>
       <c r="T111" s="3" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
       <c r="U111" s="3"/>
       <c r="V111" s="3"/>
@@ -22816,21 +22954,21 @@
       <c r="AC111" s="3"/>
       <c r="AD111" s="3"/>
       <c r="AE111" s="3" t="s">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="AF111" s="3"/>
       <c r="AG111" s="3"/>
     </row>
     <row r="112" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B112" s="8">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D112" s="3"/>
       <c r="E112" s="3" t="s">
-        <v>726</v>
+        <v>737</v>
       </c>
       <c r="F112" s="3"/>
       <c r="G112" s="3"/>
@@ -22840,7 +22978,7 @@
       <c r="K112" s="3"/>
       <c r="L112" s="3"/>
       <c r="M112" s="3" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
       <c r="N112" s="3"/>
       <c r="O112" s="3"/>
@@ -22849,7 +22987,7 @@
       <c r="R112" s="3"/>
       <c r="S112" s="3"/>
       <c r="T112" s="3" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="U112" s="3"/>
       <c r="V112" s="3"/>
@@ -22862,21 +23000,21 @@
       <c r="AC112" s="3"/>
       <c r="AD112" s="3"/>
       <c r="AE112" s="3" t="s">
-        <v>731</v>
+        <v>739</v>
       </c>
       <c r="AF112" s="3"/>
       <c r="AG112" s="3"/>
     </row>
     <row r="113" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B113" s="8">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>664</v>
+        <v>621</v>
       </c>
       <c r="D113" s="3"/>
       <c r="E113" s="3" t="s">
-        <v>729</v>
+        <v>737</v>
       </c>
       <c r="F113" s="3"/>
       <c r="G113" s="3"/>
@@ -22895,7 +23033,7 @@
       <c r="R113" s="3"/>
       <c r="S113" s="3"/>
       <c r="T113" s="3" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="U113" s="3"/>
       <c r="V113" s="3"/>
@@ -22908,21 +23046,21 @@
       <c r="AC113" s="3"/>
       <c r="AD113" s="3"/>
       <c r="AE113" s="3" t="s">
-        <v>731</v>
+        <v>739</v>
       </c>
       <c r="AF113" s="3"/>
       <c r="AG113" s="3"/>
     </row>
-    <row r="114" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B114" s="8">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>632</v>
+        <v>664</v>
       </c>
       <c r="D114" s="3"/>
       <c r="E114" s="3" t="s">
-        <v>734</v>
+        <v>741</v>
       </c>
       <c r="F114" s="3"/>
       <c r="G114" s="3"/>
@@ -22941,7 +23079,7 @@
       <c r="R114" s="3"/>
       <c r="S114" s="3"/>
       <c r="T114" s="3" t="s">
-        <v>735</v>
+        <v>742</v>
       </c>
       <c r="U114" s="3"/>
       <c r="V114" s="3"/>
@@ -22954,21 +23092,21 @@
       <c r="AC114" s="3"/>
       <c r="AD114" s="3"/>
       <c r="AE114" s="3" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="AF114" s="3"/>
       <c r="AG114" s="3"/>
     </row>
     <row r="115" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B115" s="8">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>632</v>
+        <v>688</v>
       </c>
       <c r="D115" s="3"/>
       <c r="E115" s="3" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="F115" s="3"/>
       <c r="G115" s="3"/>
@@ -22978,7 +23116,7 @@
       <c r="K115" s="3"/>
       <c r="L115" s="3"/>
       <c r="M115" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N115" s="3"/>
       <c r="O115" s="3"/>
@@ -22987,7 +23125,7 @@
       <c r="R115" s="3"/>
       <c r="S115" s="3"/>
       <c r="T115" s="3" t="s">
-        <v>738</v>
+        <v>743</v>
       </c>
       <c r="U115" s="3"/>
       <c r="V115" s="3"/>
@@ -23007,14 +23145,14 @@
     </row>
     <row r="116" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B116" s="8">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D116" s="3"/>
       <c r="E116" s="3" t="s">
-        <v>737</v>
+        <v>744</v>
       </c>
       <c r="F116" s="3"/>
       <c r="G116" s="3"/>
@@ -23024,7 +23162,7 @@
       <c r="K116" s="3"/>
       <c r="L116" s="3"/>
       <c r="M116" s="3" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
       <c r="N116" s="3"/>
       <c r="O116" s="3"/>
@@ -23033,7 +23171,7 @@
       <c r="R116" s="3"/>
       <c r="S116" s="3"/>
       <c r="T116" s="3" t="s">
-        <v>740</v>
+        <v>745</v>
       </c>
       <c r="U116" s="3"/>
       <c r="V116" s="3"/>
@@ -23046,21 +23184,21 @@
       <c r="AC116" s="3"/>
       <c r="AD116" s="3"/>
       <c r="AE116" s="3" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="AF116" s="3"/>
       <c r="AG116" s="3"/>
     </row>
     <row r="117" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B117" s="8">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>664</v>
+        <v>632</v>
       </c>
       <c r="D117" s="3"/>
       <c r="E117" s="3" t="s">
-        <v>741</v>
+        <v>746</v>
       </c>
       <c r="F117" s="3"/>
       <c r="G117" s="3"/>
@@ -23079,7 +23217,7 @@
       <c r="R117" s="3"/>
       <c r="S117" s="3"/>
       <c r="T117" s="3" t="s">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="U117" s="3"/>
       <c r="V117" s="3"/>
@@ -23099,14 +23237,14 @@
     </row>
     <row r="118" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B118" s="8">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>688</v>
+        <v>621</v>
       </c>
       <c r="D118" s="3"/>
       <c r="E118" s="3" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="F118" s="3"/>
       <c r="G118" s="3"/>
@@ -23125,7 +23263,7 @@
       <c r="R118" s="3"/>
       <c r="S118" s="3"/>
       <c r="T118" s="3" t="s">
-        <v>743</v>
+        <v>748</v>
       </c>
       <c r="U118" s="3"/>
       <c r="V118" s="3"/>
@@ -23145,14 +23283,14 @@
     </row>
     <row r="119" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B119" s="8">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>632</v>
+        <v>664</v>
       </c>
       <c r="D119" s="3"/>
       <c r="E119" s="3" t="s">
-        <v>744</v>
+        <v>749</v>
       </c>
       <c r="F119" s="3"/>
       <c r="G119" s="3"/>
@@ -23162,7 +23300,7 @@
       <c r="K119" s="3"/>
       <c r="L119" s="3"/>
       <c r="M119" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N119" s="3"/>
       <c r="O119" s="3"/>
@@ -23171,7 +23309,7 @@
       <c r="R119" s="3"/>
       <c r="S119" s="3"/>
       <c r="T119" s="3" t="s">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="U119" s="3"/>
       <c r="V119" s="3"/>
@@ -23184,21 +23322,21 @@
       <c r="AC119" s="3"/>
       <c r="AD119" s="3"/>
       <c r="AE119" s="3" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
       <c r="AF119" s="3"/>
       <c r="AG119" s="3"/>
     </row>
     <row r="120" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B120" s="8">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>632</v>
+        <v>688</v>
       </c>
       <c r="D120" s="3"/>
       <c r="E120" s="3" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="F120" s="3"/>
       <c r="G120" s="3"/>
@@ -23217,7 +23355,7 @@
       <c r="R120" s="3"/>
       <c r="S120" s="3"/>
       <c r="T120" s="3" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="U120" s="3"/>
       <c r="V120" s="3"/>
@@ -23235,16 +23373,16 @@
       <c r="AF120" s="3"/>
       <c r="AG120" s="3"/>
     </row>
-    <row r="121" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="121" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B121" s="8">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>621</v>
       </c>
       <c r="D121" s="3"/>
       <c r="E121" s="3" t="s">
-        <v>744</v>
+        <v>752</v>
       </c>
       <c r="F121" s="3"/>
       <c r="G121" s="3"/>
@@ -23263,7 +23401,7 @@
       <c r="R121" s="3"/>
       <c r="S121" s="3"/>
       <c r="T121" s="3" t="s">
-        <v>748</v>
+        <v>753</v>
       </c>
       <c r="U121" s="3"/>
       <c r="V121" s="3"/>
@@ -23283,14 +23421,14 @@
     </row>
     <row r="122" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B122" s="8">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>664</v>
+        <v>632</v>
       </c>
       <c r="D122" s="3"/>
       <c r="E122" s="3" t="s">
-        <v>749</v>
+        <v>754</v>
       </c>
       <c r="F122" s="3"/>
       <c r="G122" s="3"/>
@@ -23300,7 +23438,7 @@
       <c r="K122" s="3"/>
       <c r="L122" s="3"/>
       <c r="M122" s="3" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
       <c r="N122" s="3"/>
       <c r="O122" s="3"/>
@@ -23309,7 +23447,7 @@
       <c r="R122" s="3"/>
       <c r="S122" s="3"/>
       <c r="T122" s="3" t="s">
-        <v>750</v>
+        <v>755</v>
       </c>
       <c r="U122" s="3"/>
       <c r="V122" s="3"/>
@@ -23322,21 +23460,21 @@
       <c r="AC122" s="3"/>
       <c r="AD122" s="3"/>
       <c r="AE122" s="3" t="s">
-        <v>739</v>
+        <v>756</v>
       </c>
       <c r="AF122" s="3"/>
       <c r="AG122" s="3"/>
     </row>
     <row r="123" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B123" s="8">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>688</v>
+        <v>664</v>
       </c>
       <c r="D123" s="3"/>
       <c r="E123" s="3" t="s">
-        <v>749</v>
+        <v>754</v>
       </c>
       <c r="F123" s="3"/>
       <c r="G123" s="3"/>
@@ -23355,7 +23493,7 @@
       <c r="R123" s="3"/>
       <c r="S123" s="3"/>
       <c r="T123" s="3" t="s">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="U123" s="3"/>
       <c r="V123" s="3"/>
@@ -23368,21 +23506,21 @@
       <c r="AC123" s="3"/>
       <c r="AD123" s="3"/>
       <c r="AE123" s="3" t="s">
-        <v>739</v>
+        <v>758</v>
       </c>
       <c r="AF123" s="3"/>
       <c r="AG123" s="3"/>
     </row>
-    <row r="124" ht="30" customHeight="1" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B124" s="8">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="D124" s="3"/>
       <c r="E124" s="3" t="s">
-        <v>752</v>
+        <v>759</v>
       </c>
       <c r="F124" s="3"/>
       <c r="G124" s="3"/>
@@ -23392,7 +23530,7 @@
       <c r="K124" s="3"/>
       <c r="L124" s="3"/>
       <c r="M124" s="3" t="s">
-        <v>686</v>
+        <v>648</v>
       </c>
       <c r="N124" s="3"/>
       <c r="O124" s="3"/>
@@ -23401,7 +23539,7 @@
       <c r="R124" s="3"/>
       <c r="S124" s="3"/>
       <c r="T124" s="3" t="s">
-        <v>753</v>
+        <v>760</v>
       </c>
       <c r="U124" s="3"/>
       <c r="V124" s="3"/>
@@ -23414,21 +23552,21 @@
       <c r="AC124" s="3"/>
       <c r="AD124" s="3"/>
       <c r="AE124" s="3" t="s">
-        <v>739</v>
+        <v>761</v>
       </c>
       <c r="AF124" s="3"/>
       <c r="AG124" s="3"/>
     </row>
     <row r="125" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B125" s="8">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>632</v>
+        <v>621</v>
       </c>
       <c r="D125" s="3"/>
       <c r="E125" s="3" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="F125" s="3"/>
       <c r="G125" s="3"/>
@@ -23438,7 +23576,7 @@
       <c r="K125" s="3"/>
       <c r="L125" s="3"/>
       <c r="M125" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N125" s="3"/>
       <c r="O125" s="3"/>
@@ -23447,7 +23585,7 @@
       <c r="R125" s="3"/>
       <c r="S125" s="3"/>
       <c r="T125" s="3" t="s">
-        <v>755</v>
+        <v>762</v>
       </c>
       <c r="U125" s="3"/>
       <c r="V125" s="3"/>
@@ -23460,21 +23598,21 @@
       <c r="AC125" s="3"/>
       <c r="AD125" s="3"/>
       <c r="AE125" s="3" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="AF125" s="3"/>
       <c r="AG125" s="3"/>
     </row>
     <row r="126" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B126" s="8">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C126" s="3" t="s">
         <v>664</v>
       </c>
       <c r="D126" s="3"/>
       <c r="E126" s="3" t="s">
-        <v>754</v>
+        <v>763</v>
       </c>
       <c r="F126" s="3"/>
       <c r="G126" s="3"/>
@@ -23493,7 +23631,7 @@
       <c r="R126" s="3"/>
       <c r="S126" s="3"/>
       <c r="T126" s="3" t="s">
-        <v>757</v>
+        <v>764</v>
       </c>
       <c r="U126" s="3"/>
       <c r="V126" s="3"/>
@@ -23513,14 +23651,14 @@
     </row>
     <row r="127" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B127" s="8">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>632</v>
+        <v>688</v>
       </c>
       <c r="D127" s="3"/>
       <c r="E127" s="3" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="F127" s="3"/>
       <c r="G127" s="3"/>
@@ -23530,7 +23668,7 @@
       <c r="K127" s="3"/>
       <c r="L127" s="3"/>
       <c r="M127" s="3" t="s">
-        <v>648</v>
+        <v>686</v>
       </c>
       <c r="N127" s="3"/>
       <c r="O127" s="3"/>
@@ -23539,7 +23677,7 @@
       <c r="R127" s="3"/>
       <c r="S127" s="3"/>
       <c r="T127" s="3" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="U127" s="3"/>
       <c r="V127" s="3"/>
@@ -23552,148 +23690,10 @@
       <c r="AC127" s="3"/>
       <c r="AD127" s="3"/>
       <c r="AE127" s="3" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="AF127" s="3"/>
       <c r="AG127" s="3"/>
-    </row>
-    <row r="128" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B128" s="8">
-        <v>58</v>
-      </c>
-      <c r="C128" s="3" t="s">
-        <v>621</v>
-      </c>
-      <c r="D128" s="3"/>
-      <c r="E128" s="3" t="s">
-        <v>759</v>
-      </c>
-      <c r="F128" s="3"/>
-      <c r="G128" s="3"/>
-      <c r="H128" s="3"/>
-      <c r="I128" s="3"/>
-      <c r="J128" s="3"/>
-      <c r="K128" s="3"/>
-      <c r="L128" s="3"/>
-      <c r="M128" s="3" t="s">
-        <v>686</v>
-      </c>
-      <c r="N128" s="3"/>
-      <c r="O128" s="3"/>
-      <c r="P128" s="3"/>
-      <c r="Q128" s="3"/>
-      <c r="R128" s="3"/>
-      <c r="S128" s="3"/>
-      <c r="T128" s="3" t="s">
-        <v>762</v>
-      </c>
-      <c r="U128" s="3"/>
-      <c r="V128" s="3"/>
-      <c r="W128" s="3"/>
-      <c r="X128" s="3"/>
-      <c r="Y128" s="3"/>
-      <c r="Z128" s="3"/>
-      <c r="AA128" s="3"/>
-      <c r="AB128" s="3"/>
-      <c r="AC128" s="3"/>
-      <c r="AD128" s="3"/>
-      <c r="AE128" s="3" t="s">
-        <v>758</v>
-      </c>
-      <c r="AF128" s="3"/>
-      <c r="AG128" s="3"/>
-    </row>
-    <row r="129" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B129" s="8">
-        <v>59</v>
-      </c>
-      <c r="C129" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D129" s="3"/>
-      <c r="E129" s="3" t="s">
-        <v>763</v>
-      </c>
-      <c r="F129" s="3"/>
-      <c r="G129" s="3"/>
-      <c r="H129" s="3"/>
-      <c r="I129" s="3"/>
-      <c r="J129" s="3"/>
-      <c r="K129" s="3"/>
-      <c r="L129" s="3"/>
-      <c r="M129" s="3" t="s">
-        <v>686</v>
-      </c>
-      <c r="N129" s="3"/>
-      <c r="O129" s="3"/>
-      <c r="P129" s="3"/>
-      <c r="Q129" s="3"/>
-      <c r="R129" s="3"/>
-      <c r="S129" s="3"/>
-      <c r="T129" s="3" t="s">
-        <v>764</v>
-      </c>
-      <c r="U129" s="3"/>
-      <c r="V129" s="3"/>
-      <c r="W129" s="3"/>
-      <c r="X129" s="3"/>
-      <c r="Y129" s="3"/>
-      <c r="Z129" s="3"/>
-      <c r="AA129" s="3"/>
-      <c r="AB129" s="3"/>
-      <c r="AC129" s="3"/>
-      <c r="AD129" s="3"/>
-      <c r="AE129" s="3" t="s">
-        <v>758</v>
-      </c>
-      <c r="AF129" s="3"/>
-      <c r="AG129" s="3"/>
-    </row>
-    <row r="130" spans="2:33" x14ac:dyDescent="0.25">
-      <c r="B130" s="8">
-        <v>60</v>
-      </c>
-      <c r="C130" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="D130" s="3"/>
-      <c r="E130" s="3" t="s">
-        <v>763</v>
-      </c>
-      <c r="F130" s="3"/>
-      <c r="G130" s="3"/>
-      <c r="H130" s="3"/>
-      <c r="I130" s="3"/>
-      <c r="J130" s="3"/>
-      <c r="K130" s="3"/>
-      <c r="L130" s="3"/>
-      <c r="M130" s="3" t="s">
-        <v>686</v>
-      </c>
-      <c r="N130" s="3"/>
-      <c r="O130" s="3"/>
-      <c r="P130" s="3"/>
-      <c r="Q130" s="3"/>
-      <c r="R130" s="3"/>
-      <c r="S130" s="3"/>
-      <c r="T130" s="3" t="s">
-        <v>765</v>
-      </c>
-      <c r="U130" s="3"/>
-      <c r="V130" s="3"/>
-      <c r="W130" s="3"/>
-      <c r="X130" s="3"/>
-      <c r="Y130" s="3"/>
-      <c r="Z130" s="3"/>
-      <c r="AA130" s="3"/>
-      <c r="AB130" s="3"/>
-      <c r="AC130" s="3"/>
-      <c r="AD130" s="3"/>
-      <c r="AE130" s="3" t="s">
-        <v>758</v>
-      </c>
-      <c r="AF130" s="3"/>
-      <c r="AG130" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="409">
@@ -23740,6 +23740,18 @@
     <mergeCell ref="L25:AG25"/>
     <mergeCell ref="B27:AG27"/>
     <mergeCell ref="B28:AG28"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="G45:O45"/>
+    <mergeCell ref="P45:V45"/>
+    <mergeCell ref="W45:AG45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="G46:O46"/>
+    <mergeCell ref="P46:V46"/>
+    <mergeCell ref="W46:AG46"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="G47:O47"/>
+    <mergeCell ref="P47:V47"/>
+    <mergeCell ref="W47:AG47"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="G48:O48"/>
     <mergeCell ref="P48:V48"/>
@@ -23756,19 +23768,16 @@
     <mergeCell ref="G51:O51"/>
     <mergeCell ref="P51:V51"/>
     <mergeCell ref="W51:AG51"/>
-    <mergeCell ref="B52:F52"/>
-    <mergeCell ref="G52:O52"/>
-    <mergeCell ref="P52:V52"/>
-    <mergeCell ref="W52:AG52"/>
-    <mergeCell ref="B53:F53"/>
-    <mergeCell ref="G53:O53"/>
-    <mergeCell ref="P53:V53"/>
-    <mergeCell ref="W53:AG53"/>
-    <mergeCell ref="B54:F54"/>
-    <mergeCell ref="G54:O54"/>
-    <mergeCell ref="P54:V54"/>
-    <mergeCell ref="W54:AG54"/>
-    <mergeCell ref="B56:AG56"/>
+    <mergeCell ref="B53:AG53"/>
+    <mergeCell ref="B54:H54"/>
+    <mergeCell ref="I54:W54"/>
+    <mergeCell ref="X54:AG54"/>
+    <mergeCell ref="B55:H55"/>
+    <mergeCell ref="I55:W55"/>
+    <mergeCell ref="X55:AG55"/>
+    <mergeCell ref="B56:H56"/>
+    <mergeCell ref="I56:W56"/>
+    <mergeCell ref="X56:AG56"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="I57:W57"/>
     <mergeCell ref="X57:AG57"/>
@@ -23790,17 +23799,23 @@
     <mergeCell ref="B63:H63"/>
     <mergeCell ref="I63:W63"/>
     <mergeCell ref="X63:AG63"/>
-    <mergeCell ref="B64:H64"/>
-    <mergeCell ref="I64:W64"/>
-    <mergeCell ref="X64:AG64"/>
-    <mergeCell ref="B65:H65"/>
-    <mergeCell ref="I65:W65"/>
-    <mergeCell ref="X65:AG65"/>
-    <mergeCell ref="B66:H66"/>
-    <mergeCell ref="I66:W66"/>
-    <mergeCell ref="X66:AG66"/>
-    <mergeCell ref="B67:AG67"/>
-    <mergeCell ref="B69:AG69"/>
+    <mergeCell ref="B64:AG64"/>
+    <mergeCell ref="B66:AG66"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="E67:L67"/>
+    <mergeCell ref="M67:S67"/>
+    <mergeCell ref="T67:AD67"/>
+    <mergeCell ref="AE67:AG67"/>
+    <mergeCell ref="C68:D68"/>
+    <mergeCell ref="E68:L68"/>
+    <mergeCell ref="M68:S68"/>
+    <mergeCell ref="T68:AD68"/>
+    <mergeCell ref="AE68:AG68"/>
+    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="E69:L69"/>
+    <mergeCell ref="M69:S69"/>
+    <mergeCell ref="T69:AD69"/>
+    <mergeCell ref="AE69:AG69"/>
     <mergeCell ref="C70:D70"/>
     <mergeCell ref="E70:L70"/>
     <mergeCell ref="M70:S70"/>
@@ -24091,21 +24106,6 @@
     <mergeCell ref="M127:S127"/>
     <mergeCell ref="T127:AD127"/>
     <mergeCell ref="AE127:AG127"/>
-    <mergeCell ref="C128:D128"/>
-    <mergeCell ref="E128:L128"/>
-    <mergeCell ref="M128:S128"/>
-    <mergeCell ref="T128:AD128"/>
-    <mergeCell ref="AE128:AG128"/>
-    <mergeCell ref="C129:D129"/>
-    <mergeCell ref="E129:L129"/>
-    <mergeCell ref="M129:S129"/>
-    <mergeCell ref="T129:AD129"/>
-    <mergeCell ref="AE129:AG129"/>
-    <mergeCell ref="C130:D130"/>
-    <mergeCell ref="E130:L130"/>
-    <mergeCell ref="M130:S130"/>
-    <mergeCell ref="T130:AD130"/>
-    <mergeCell ref="AE130:AG130"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <drawing r:id="rId1"/>

</xml_diff>